<commit_message>
save repo before changing scale logic
</commit_message>
<xml_diff>
--- a/data/results.xlsx
+++ b/data/results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\pycharm_projects\network_simulations\thesis\throughput_upperbound\simulations\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26709424-1105-4BFA-92D8-83CD9A26B3F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D4B806-776F-4C44-B1C2-70E30A44D49D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{721E2542-CFD3-F545-91FB-44EA0C7E0544}"/>
+    <workbookView xWindow="-130" yWindow="-130" windowWidth="19460" windowHeight="10340" activeTab="3" xr2:uid="{721E2542-CFD3-F545-91FB-44EA0C7E0544}"/>
   </bookViews>
   <sheets>
     <sheet name="throughtput" sheetId="2" r:id="rId1"/>
@@ -4595,6 +4595,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C41AEE1E-4CBB-415F-95F8-165D4B6A1E64}">
   <dimension ref="A1:O52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -4708,7 +4712,7 @@
         <v>198</v>
       </c>
       <c r="E5">
-        <f t="shared" ref="E3:E6" si="0">D5/J5</f>
+        <f t="shared" ref="E5:E6" si="0">D5/J5</f>
         <v>60.96507454074321</v>
       </c>
       <c r="I5" t="s">
@@ -4880,7 +4884,7 @@
         <v>23</v>
       </c>
       <c r="E12">
-        <f t="shared" ref="E7:E52" si="2">D12/J12</f>
+        <f t="shared" ref="E12:E52" si="2">D12/J12</f>
         <v>62.246433339000234</v>
       </c>
       <c r="G12" s="2"/>

</xml_diff>